<commit_message>
fix: Corrige ubicacion de textos en el Excel
</commit_message>
<xml_diff>
--- a/semana_5/DOD_Completado.xlsx
+++ b/semana_5/DOD_Completado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\Adolfo\Desktop\ingenieria de sotfware\s5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE0DC7-DD1C-45D8-8947-5022D513C8F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9C454A-C629-4473-BE6D-071EAAC854F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
   <si>
     <t>DEFINICION DEL  DOD</t>
   </si>
@@ -208,9 +208,6 @@
   </si>
   <si>
     <t>COMPONENTE 3</t>
-  </si>
-  <si>
-    <t>COMPONENTE 4</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -661,13 +658,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>COMPONENTE 1</c:v>
+                  <c:v>Vista Búsqueda</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>COMPONENTE 2</c:v>
+                  <c:v>Vista Reserva</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>COMPONENTE 3</c:v>
+                  <c:v>Panel Administrador</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1266,16 +1263,13 @@
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="16" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="18"/>
       <c r="I3" s="7">
         <f>SUM(D2:D5)/12</f>
         <v>1</v>
-      </c>
-      <c r="K3" t="s">
-        <v>22</v>
       </c>
       <c r="L3" s="8" t="s">
         <v>10</v>
@@ -1301,16 +1295,13 @@
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="16" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="18"/>
       <c r="I4" s="7">
         <f>SUM(D6:D9)/12</f>
         <v>1</v>
-      </c>
-      <c r="K4" t="s">
-        <v>23</v>
       </c>
       <c r="L4" s="9">
         <v>0</v>
@@ -1336,7 +1327,7 @@
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="16" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G5" s="17"/>
       <c r="H5" s="18"/>
@@ -1344,9 +1335,6 @@
         <f>SUM(D10,D13)/6</f>
         <v>1</v>
       </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="6" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="24"/>
@@ -1361,16 +1349,13 @@
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="16" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G6" s="17"/>
       <c r="H6" s="18"/>
       <c r="I6" s="7">
         <f>SUM(D14,D17)/6</f>
         <v>1</v>
-      </c>
-      <c r="K6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1384,7 +1369,7 @@
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7" s="17"/>
       <c r="H7" s="18"/>
@@ -1476,7 +1461,7 @@
     <row r="14" spans="1:15" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24"/>
       <c r="B14" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>4</v>
@@ -2575,7 +2560,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -3623,6 +3608,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010070BFDEA41A5D8B46AA5DA2E2389CBE4E" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="672700c7c1e39a78a362f54b21ce1efa">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d0daa353-f819-43d1-badf-ce69fea8800d" xmlns:ns3="edc1eb1c-f9b5-429a-a0ce-702847a0aa2d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3db37e5c6f54565a9911855e2c96e577" ns2:_="" ns3:_="">
     <xsd:import namespace="d0daa353-f819-43d1-badf-ce69fea8800d"/>
@@ -3877,15 +3871,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A26DB7C-878E-46E5-89F2-71019BF99099}">
   <ds:schemaRefs>
@@ -3898,6 +3883,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47A3290B-B6C1-4BEF-B4D8-BE863B785917}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81288DC1-A1A5-4A8F-86BC-34BD167F9197}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3914,12 +3907,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47A3290B-B6C1-4BEF-B4D8-BE863B785917}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>